<commit_message>
Uses LLM ollama cloud for triple extraction
</commit_message>
<xml_diff>
--- a/evaluation/evaluation_reports/2025-04-07/overview_2025-04-07.xlsx
+++ b/evaluation/evaluation_reports/2025-04-07/overview_2025-04-07.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/piek/Desktop/d-Leolani/cltl-knowledgeextraction/examples/evaluation_reports/2025-04-07/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/piek/Desktop/d-Leolani/cltl-knowledgeextraction/evaluation/evaluation_reports/2025-04-07/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8113A133-4809-434B-97CA-1CC561A865BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E7FD2CC3-9AFB-5F45-913B-9251DB1BDBCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6380" yWindow="3600" windowWidth="33520" windowHeight="18640" activeTab="2" xr2:uid="{F990004E-9E21-8648-8818-D1DDDDEA31B1}"/>
+    <workbookView xWindow="70100" yWindow="4480" windowWidth="33520" windowHeight="18640" activeTab="2" xr2:uid="{F990004E-9E21-8648-8818-D1DDDDEA31B1}"/>
   </bookViews>
   <sheets>
     <sheet name="overview_2025-04-07" sheetId="3" r:id="rId1"/>
@@ -394,7 +394,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -574,6 +574,12 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -735,10 +741,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -4802,10 +4809,10 @@
       <c r="K2" t="s">
         <v>55</v>
       </c>
-      <c r="L2">
+      <c r="L2" s="3">
         <v>14</v>
       </c>
-      <c r="M2">
+      <c r="M2" s="3">
         <v>13</v>
       </c>
       <c r="N2">
@@ -4822,7 +4829,7 @@
       <c r="F3" t="s">
         <v>56</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="3">
         <v>18</v>
       </c>
       <c r="K3" t="s">
@@ -4833,16 +4840,16 @@
       <c r="A4" t="s">
         <v>57</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="3">
         <v>57</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="3">
         <v>28</v>
       </c>
       <c r="F4" t="s">
         <v>57</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="3">
         <v>35</v>
       </c>
       <c r="H4">
@@ -4851,7 +4858,7 @@
       <c r="K4" t="s">
         <v>57</v>
       </c>
-      <c r="L4">
+      <c r="L4" s="3">
         <v>13</v>
       </c>
       <c r="M4">
@@ -4879,7 +4886,7 @@
       <c r="A7" t="s">
         <v>59</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="3">
         <v>29</v>
       </c>
       <c r="F7" t="s">
@@ -4891,7 +4898,7 @@
       <c r="K7" t="s">
         <v>59</v>
       </c>
-      <c r="N7">
+      <c r="N7" s="3">
         <v>15</v>
       </c>
     </row>
@@ -4899,7 +4906,7 @@
       <c r="A8" t="s">
         <v>60</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="3">
         <v>13</v>
       </c>
       <c r="F8" t="s">
@@ -4919,7 +4926,7 @@
       <c r="A9" t="s">
         <v>61</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="3">
         <v>10</v>
       </c>
       <c r="F9" t="s">
@@ -4933,7 +4940,7 @@
       <c r="A10" t="s">
         <v>62</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="3">
         <v>18</v>
       </c>
       <c r="F10" t="s">
@@ -4947,13 +4954,13 @@
       <c r="A11" t="s">
         <v>63</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="3">
         <v>23</v>
       </c>
       <c r="F11" t="s">
         <v>63</v>
       </c>
-      <c r="I11">
+      <c r="I11" s="3">
         <v>12</v>
       </c>
       <c r="K11" t="s">

</xml_diff>